<commit_message>
Added CMSIS. Added clock setup code for PLL1, used for MCU core and busses. Added code for enabling the peripherials used by Etherbridge. Added GPIO initialsation code and pinout config table.
</commit_message>
<xml_diff>
--- a/HW-Doc/MCU Pinout LQFP48.xlsx
+++ b/HW-Doc/MCU Pinout LQFP48.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Fki\Documents\Projekte\Etherbridge_custom\HW-Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DEB8657-D779-49EE-B76F-AE397BA0E706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{112E1323-90FC-4D4C-A3BC-AEB83AE3A61C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2BCB3841-5261-458E-B6D1-67570C2DFED8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="119">
   <si>
     <t>PinNr</t>
   </si>
@@ -359,9 +359,6 @@
     <t>Program Enable</t>
   </si>
   <si>
-    <t>Chip Select</t>
-  </si>
-  <si>
     <t>WZ_CLK</t>
   </si>
   <si>
@@ -390,6 +387,12 @@
   </si>
   <si>
     <t>MCU Pin</t>
+  </si>
+  <si>
+    <t>93LC86 Chip Select</t>
+  </si>
+  <si>
+    <t>USART1_RX</t>
   </si>
 </sst>
 </file>
@@ -950,7 +953,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C1" s="20" t="s">
         <v>76</v>
@@ -1402,7 +1405,7 @@
         <v>67</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="E29" s="11" t="s">
         <v>82</v>
@@ -1416,10 +1419,10 @@
         <v>38</v>
       </c>
       <c r="C30" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="D30" s="9" t="s">
         <v>108</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>109</v>
       </c>
       <c r="E30" s="9" t="s">
         <v>39</v>
@@ -1433,7 +1436,7 @@
         <v>40</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D31" s="15" t="s">
         <v>36</v>
@@ -1450,10 +1453,10 @@
         <v>41</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>19</v>
+        <v>118</v>
       </c>
       <c r="E32" s="15" t="s">
         <v>17</v>
@@ -1467,7 +1470,7 @@
         <v>42</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D33" s="19" t="s">
         <v>43</v>
@@ -1484,7 +1487,7 @@
         <v>45</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D34" s="19" t="s">
         <v>46</v>
@@ -1504,7 +1507,7 @@
         <v>48</v>
       </c>
       <c r="D35" s="17" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E35" s="17" t="s">
         <v>39</v>
@@ -1547,7 +1550,7 @@
         <v>50</v>
       </c>
       <c r="D38" s="17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E38" s="17" t="s">
         <v>39</v>
@@ -1581,7 +1584,7 @@
         <v>69</v>
       </c>
       <c r="D40" s="17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E40" s="17" t="s">
         <v>39</v>

</xml_diff>